<commit_message>
Updated Theme and Made it have a unique design
</commit_message>
<xml_diff>
--- a/Income Statement and distribution.xlsx
+++ b/Income Statement and distribution.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\xammp\htdocs\schoolprojectt\SmartStudyProV2.3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5D38FA-1596-4C0C-85BB-E4BDD5EA6E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2BFFC81-3C56-41B1-97B5-6A82DF085595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A9249DB2-D755-4C5E-BBBA-849229C05261}"/>
   </bookViews>
@@ -250,7 +250,7 @@
                 <c:formatCode>_("USh"* #,##0_);_("USh"* \(#,##0\);_("USh"* "-"_);_(@_)</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>120000</c:v>
+                  <c:v>150000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -641,7 +641,7 @@
                 <c:formatCode>_("USh"* #,##0_);_("USh"* \(#,##0\);_("USh"* "-"_);_(@_)</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>480000</c:v>
+                  <c:v>750000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1830,11 +1830,11 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>1200000</v>
+        <v>1500000</v>
       </c>
       <c r="B3" s="1">
         <f>A3*0.1</f>
-        <v>120000</v>
+        <v>150000</v>
       </c>
       <c r="C3" s="1">
         <v>150000</v>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="I3" s="1">
         <f>A3-B3-C3-D3-E3-F3-G3-H3</f>
-        <v>480000</v>
+        <v>750000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>